<commit_message>
feat(F-NAR-009): DIF.COR 001-07/08 et 002-01–06
Ouvertures monde d’abord (herbe coupée, cloche, gouttière, feuille
à la grille, gymnase, dalle, fontaine, horloge). Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-07.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-07.xlsx
@@ -1333,7 +1333,8 @@
 narrateur|Un oiseau picore près de la haie.
 narrateur|En ce moment, Victorina marche vers le bac.
 maman|Tu as vu le banc chaud, Victorina ?
-enfant-f|Oui, maman. Il est chaud.
+enfant-f|Oui, maman.
+enfant-f|Il est chaud.
 narrateur|Victorina touche le bois du banc.
 narrateur|Le bois est lisse et un peu rugueux.
 narrateur|Elle glisse l'aiguille de pin dans sa poche.
@@ -1342,7 +1343,8 @@
 narrateur|Aniss est plus grand.
 narrateur|Victorina est plus petite.
 narrateur|Ils ont des tailles différentes.
-maman|Aniss est là. Tu veux l'inviter ?
+maman|Aniss est là.
+maman|Tu veux l'inviter ?
 enfant-f|Tu veux jouer ?
 copain|Oui.
 narrateur|Ils vont près du bac à sable.
@@ -1351,7 +1353,8 @@
 narrateur|Aniss porte un gros seau bleu.
 narrateur|Victorina porte un petit seau jaune.
 narrateur|Les seaux n'ont pas la même taille.
-maman|On joue ensemble. On reste gentils.
+maman|On joue ensemble.
+maman|On reste gentils.
 narrateur|Victorina verse du sable.
 narrateur|Ça fait un petit bruit de pluie.
 narrateur|Aniss lisse le tas avec la main.
@@ -1360,7 +1363,8 @@
 copain|Avec une tour.
 narrateur|Victorina pose un caillou gris sur le toit.
 narrateur|Aniss pose la feuille jaune à côté.
-maman|Bravo. Vous construisez ensemble.
+maman|Bravo.
+maman|Vous construisez ensemble.
 maman|Petit ou grand, on peut jouer ensemble.
 narrateur|Aniss sort une corde du sac.
 narrateur|La corde est un peu haute.
@@ -1369,7 +1373,8 @@
 narrateur|Aniss tient l'autre bout.
 narrateur|Ils sautent un peu.
 narrateur|Puis ils sautent ensemble.
-maman|Vous sautez ensemble. C'est ça.
+maman|Vous sautez ensemble.
+maman|C'est ça.
 maman|Vous avez des tailles différentes.
 maman|Et vous jouez ensemble.
 narrateur|Victorina rit du jeu.
@@ -1378,7 +1383,8 @@
 narrateur|Le cerceau rouge attend dans l'herbe.
 narrateur|Le soleil tape un peu le banc.
 maman|Le sable est doux, hein ?
-enfant-f|Oui. Il est doux.</t>
+enfant-f|Oui.
+enfant-f|Il est doux.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1743,15 +1749,18 @@
 narrateur|Aniss a dit oui.
 narrateur|Ils ont des tailles différentes.
 narrateur|Ils jouent ensemble près du bac.
-maman|Bravo, Victorina. Tu as fait du bon travail.
-maman|Vous avez invité. Vous jouez.
+maman|Bravo, Victorina.
+maman|Tu as fait du bon travail.
+maman|Vous avez invité.
+maman|Vous jouez.
 narrateur|Victorina reprend le petit seau.
 narrateur|Aniss reprend le gros seau.
 narrateur|Ils ajoutent une porte au château.
 enfant-f|La porte est là.
 copain|Je mets un pont.
 maman|Le pont est solide ?
-copain|Oui. Il tient.
+copain|Oui.
+copain|Il tient.
 narrateur|Victorina tapote le pont avec le doigt.
 narrateur|Le sable tient.</t>
         </is>
@@ -1923,11 +1932,13 @@
 narrateur|Le cerceau rouge rentre dans le sac.
 maman|Tu as fini de ranger le seau ?
 enfant-f|Oui, maman.
-maman|Merci. Bravo.
+maman|Merci.
+maman|Bravo.
 narrateur|Victorina sort l'aiguille de pin.
 narrateur|Elle la pose sur le banc chaud.
 narrateur|Le parc sent encore l'herbe.
-maman|On rentre. Le château reste un peu.
+maman|On rentre.
+maman|Le château reste un peu.
 enfant-f|Au revoir, château.
 copain|Au revoir.</t>
         </is>
@@ -2099,7 +2110,8 @@
         <is>
           <t>enfant-f|On a joué ensemble.
 maman|Petit ou grand, on peut jouer ensemble.
-maman|Bravo. C'était du bon travail.
+maman|Bravo.
+maman|C'était du bon travail.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -2122,7 +2134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2165,6 +2177,34 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-07 Les caisses d'oranges de Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-07.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour après le marché</t>
+          <t>cour après le marché, figue, pierre, caisses</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, Aniss, maman</t>
+          <t>Victorina, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut une boutique d'oranges dans la cour. L'enseigne est trop haute. Elle invite Aniss. Ils ont des tailles différentes. Ils ouvrent le magasin, ensemble.</t>
+          <t>Un jus collant tient sur la pierre. Sur la peau, un éclat de figue luit. Cour après le marché, caisses, figuier. Victorina veut la boutique d'oranges maintenant. Elle tire trop vite, enseigne trop haute. Aniss : attends. L'éclat glisse. Elle refuse de foncer, invite. Aniss regarde, tend le bras. Merci vécu. L'orange file sous la pile. Elle refuse, se glisse. Un éclat de figue reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La figue trop mûre a taché la pierre. Une odeur d'orange reste dans la cour. Les caisses du marché sont empilées. Le store de toile claque un peu. Une guêpe tourne près d'une écorce. L'ombre du figuier est fraîche. Maman pose un panier contre le mur. Tu as vu les caisses, Victorina ? Oui, maman. Elles sentent encore l'orange. Il en reste trois, au fond. En ce moment, Victorina tire une caisse. Le bois est rêche et chaud. Je veux une boutique. Une boutique d'oranges. Tu veux un magasin, ici ? Oui. Avec une enseigne. Victorina a un papier. Dessus, une orange un peu penchée. Elle veut l'accrocher tout en haut. La caisse du haut est trop haute. Ses doigts touchent seulement le bord. Oh. Je n'arrive pas. Aniss arrive dans la cour. Ses sandales font un bruit sec. Aniss est plus grand. Victorina est plus petite. Ils ont des tailles différentes. Aniss est là. Tu veux l'inviter ? Aniss, tu veux la boutique ? Oui. Ils poussent deux caisses. Aniss porte la grande. Victorina pousse la petite. On peut jouer ensemble. Vous jouez ensemble ? Oui. Oui. Le papier attend encore par terre. L'enseigne, Aniss. Elle va tout en haut.</t>
+          <t>Un jus collant tient sur la pierre. C'est sucré, papa. Tu le sens, sous le doigt ? Oui, un peu chaud. Sur la peau, un éclat de figue luit. Il brille, maman. C'est le soleil, sur la figue ? Oui, un petit point. L'ombre du figuier est fraîche. Ça sent l'orange. Les caisses viennent du marché. Oui, papa. Le store de toile claque un peu. Une guêpe tourne près d'une écorce. Elle tourne, là. On reste près des caisses ? Oui, maman. Maman pose un panier contre le mur. Trois oranges dorment au fond. Je les vois. Tu les comptes, Victorina ? Trois. Je veux une boutique, maintenant ! Une boutique d'oranges, ici ? Oui. Avec une enseigne. Victorina a un papier. Dessus, une orange un peu penchée. Elle va tout en haut ! En ce moment, Victorina tire une caisse trop vite. Le bois est rêche et chaud. La pile penche. Oh. Ses doigts touchent seulement le bord. Je n'arrive pas. L'éclat de figue glisse sur la pierre. Il part. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Aniss arrive dans la cour. Ses sandales font un bruit sec. Aniss ! La boutique, tout de suite ! Attends. Aniss reste près du mur. Oh. Tu parles à Aniss, Victorina ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le store. Personne n'entend la fin. Victorina referme la bouche, un instant. Le papier reste par terre, un peu lourd.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La figue trop mûre a taché la pierre. Une odeur d'orange reste dans la cour. Les caisses du marché sont empilées. Le store de toile claque un peu. Une guêpe tourne près d'une écorce. L'ombre du figuier est fraîche. Maman pose un panier contre le mur. Tu as vu les caisses, Victorina ? Oui, maman. Elles sentent encore l'orange. Il en reste trois, au fond. En ce moment, Victorina tire une caisse. Le bois est rêche et chaud. Je veux une boutique. Une boutique d'oranges. Tu veux un magasin, ici ? Oui. Avec une enseigne. Victorina a un papier. Dessus, une orange un peu penchée. Elle veut l'accrocher tout en haut. La caisse du haut est trop haute. Ses doigts touchent seulement le bord. Oh. Je n'arrive pas. Aniss arrive dans la cour. Ses sandales font un bruit sec. Aniss est plus grand. Victorina est plus petite. Ils ont des tailles différentes. Aniss est là. Tu veux l'inviter ? Aniss, tu veux la boutique ? Oui. Ils poussent deux caisses. Aniss porte la grande. Victorina pousse la petite. On peut jouer ensemble. Vous jouez ensemble ? Oui. Oui. Le papier attend encore par terre. L'enseigne, Aniss. Elle va tout en haut.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un jus collant tient sur la pierre. C'est sucré, papa. Tu le sens, sous le doigt ? Oui, un peu chaud. Sur la peau, un &lt;emphasis level="moderate"&gt;éclat de figue&lt;/emphasis&gt; luit. Il brille, maman. C'est le soleil, sur la figue ? Oui, un petit point. L'ombre du figuier est fraîche. Ça sent l'orange. Les caisses viennent du marché. Oui, papa. Le store de toile claque un peu. Une guêpe tourne près d'une écorce. Elle tourne, là. On reste près des caisses ? Oui, maman. Maman pose un panier contre le mur. Trois oranges dorment au fond. Je les vois. Tu les comptes, Victorina ? Trois. Je veux une boutique, maintenant ! Une boutique d'oranges, ici ? Oui. Avec une enseigne. Victorina a un papier. Dessus, une orange un peu penchée. Elle va tout en haut ! En ce moment, Victorina tire une caisse trop vite. Le bois est rêche et chaud. La pile penche. Oh. Ses doigts touchent seulement le bord. Je n'arrive pas. L'éclat de figue glisse sur la pierre. Il part. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Aniss arrive dans la cour. Ses sandales font un bruit sec. Aniss ! La boutique, tout de suite ! Attends. Aniss reste près du mur. Oh. Tu parles à Aniss, Victorina ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le store. Personne n'entend la fin. Victorina referme la bouche, un instant. Le papier reste par terre, un peu lourd.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Coralie est au parc avec maman. Hippolyte arrive avec un cerceau. Hippolyte est plus grand. Coralie est plus petite. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Maman sourit. Coralie va vers Hippolyte. Elle l'invite. Coralie dit : tu veux jouer ? Hippolyte dit : oui. Ils jouent ensemble près du bac à sable. Hippolyte porte un gros seau. Coralie porte un petit seau. Les tailles différentes restent là. On ne commente pas le corps. On joue. Hippolyte baisse un peu la corde. Coralie tient un bout. Ils sautent un peu. Puis ils sautent ensemble. Maman dit : petit ou grand, on peut jouer ensemble. Coralie verse du sable. Hippolyte lisse le tas. Maman dit : vous avez des tailles différentes. Et vous jouez ensemble. [pause]</t>
+          <t>Un jus collant tient sur la pierre. C'est sucré, papa. Tu le sens, sous le doigt ? Oui, un peu chaud. Sur la peau, un &lt;emphasis&gt;éclat de figue&lt;/emphasis&gt; luit. Il brille, maman. C'est le soleil, sur la figue ? Oui, un petit point. L'ombre du figuier est fraîche. Ça sent l'orange. Les caisses viennent du marché. Oui, papa. Le store de toile claque un peu. Une guêpe tourne près d'une écorce. Elle tourne, là. On reste près des caisses ? Oui, maman. Maman pose un panier contre le mur. Trois oranges dorment au fond. Je les vois. Tu les comptes, Victorina ? Trois. Je veux une boutique, maintenant ! Une boutique d'oranges, ici ? Oui. Avec une enseigne. Victorina a un papier. Dessus, une orange un peu penchée. Elle va tout en haut ! En ce moment, Victorina tire une caisse trop vite. Le bois est rêche et chaud. La pile penche. Oh. Ses doigts touchent seulement le bord. Je n'arrive pas. L'éclat de figue glisse sur la pierre. Il part. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Aniss arrive dans la cour. Ses sandales font un bruit sec. Aniss ! La boutique, tout de suite ! Attends. Aniss reste près du mur. Oh. Tu parles à Aniss, Victorina ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le store. Personne n'entend la fin. Victorina referme la bouche, un instant. Le papier reste par terre, un peu lourd. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de figue</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,58 +1321,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_boutique_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La figue trop mûre a taché la pierre.
-narrateur|Une odeur d'orange reste dans la cour.
-narrateur|Les caisses du marché sont empilées.
+          <t>narrateur|Un jus collant tient sur la pierre.
+enfant-f|C'est sucré, papa.
+papa|Tu le sens, sous le doigt ?
+enfant-f|Oui, un peu chaud.
+narrateur|Sur la peau, un éclat de figue luit.
+enfant-f|Il brille, maman.
+maman|C'est le soleil, sur la figue ?
+enfant-f|Oui, un petit point.
+narrateur|L'ombre du figuier est fraîche.
+enfant-f|Ça sent l'orange.
+papa|Les caisses viennent du marché.
+enfant-f|Oui, papa.
 narrateur|Le store de toile claque un peu.
 narrateur|Une guêpe tourne près d'une écorce.
-narrateur|L'ombre du figuier est fraîche.
+enfant-f|Elle tourne, là.
+maman|On reste près des caisses ?
+enfant-f|Oui, maman.
 narrateur|Maman pose un panier contre le mur.
-maman|Tu as vu les caisses, Victorina ?
-enfant-f|Oui, maman.
-enfant-f|Elles sentent encore l'orange.
-maman|Il en reste trois, au fond.
-narrateur|En ce moment, Victorina tire une caisse.
-narrateur|Le bois est rêche et chaud.
-enfant-f|Je veux une boutique.
-enfant-f|Une boutique d'oranges.
-maman|Tu veux un magasin, ici ?
+narrateur|Trois oranges dorment au fond.
+enfant-f|Je les vois.
+papa|Tu les comptes, Victorina ?
+enfant-f|Trois.
+enfant-f|Je veux une boutique, maintenant !
+papa|Une boutique d'oranges, ici ?
 enfant-f|Oui.
 enfant-f|Avec une enseigne.
 narrateur|Victorina a un papier.
 narrateur|Dessus, une orange un peu penchée.
-narrateur|Elle veut l'accrocher tout en haut.
-narrateur|La caisse du haut est trop haute.
+enfant-f|Elle va tout en haut !
+narrateur|En ce moment, Victorina tire une caisse trop vite.
+narrateur|Le bois est rêche et chaud.
+narrateur|La pile penche.
+enfant-f|Oh.
 narrateur|Ses doigts touchent seulement le bord.
-enfant-f|Oh.
 enfant-f|Je n'arrive pas.
+narrateur|L'éclat de figue glisse sur la pierre.
+enfant-f|Il part.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
 narrateur|Aniss arrive dans la cour.
 narrateur|Ses sandales font un bruit sec.
-narrateur|Aniss est plus grand.
-narrateur|Victorina est plus petite.
-narrateur|Ils ont des tailles différentes.
-maman|Aniss est là.
-maman|Tu veux l'inviter ?
-enfant-f|Aniss, tu veux la boutique ?
-copain|Oui.
-narrateur|Ils poussent deux caisses.
-narrateur|Aniss porte la grande.
-narrateur|Victorina pousse la petite.
-maman|On peut jouer ensemble.
-maman|Vous jouez ensemble ?
-enfant-f|Oui.
-copain|Oui.
-narrateur|Le papier attend encore par terre.
-enfant-f|L'enseigne, Aniss.
-enfant-f|Elle va tout en haut.</t>
+enfant-f|Aniss !
+enfant-f|La boutique, tout de suite !
+copain|Attends.
+narrateur|Aniss reste près du mur.
+enfant-f|Oh.
+papa|Tu parles à Aniss, Victorina ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+narrateur|La phrase se perd dans le store.
+narrateur|Personne n'entend la fin.
+narrateur|Victorina referme la bouche, un instant.
+narrateur|Le papier reste par terre, un peu lourd.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>figue,caisse</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1417,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina invite Aniss. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina invite &lt;emphasis level="moderate"&gt;Aniss&lt;/emphasis&gt;. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Coralie invite Hippolyte. Que font-ils ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina invite &lt;emphasis&gt;Aniss&lt;/emphasis&gt;. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1472,7 +1485,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1483,7 +1496,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1498,34 +1511,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Aniss</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,17 +1557,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_invite_aniss_ils_jouent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1583,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss tend le bras. Il pose le papier sur la caisse. L'orange dessinée regarde la cour. La boutique est ouverte ! Bravo, Aniss. Tu as mis l'enseigne. Victorina s'assoit derrière la petite caisse. C'est le comptoir. Elle aligne les trois oranges. Une orange roule sous la pile. Elle est partie. Je ne la vois plus. Victorina se glisse près du bois. Elle est plus petite. Elle attrape l'orange. Te voilà. Chacun aide, à sa taille. Vous jouez ensemble. Maman prend une pièce imaginaire. Une orange, s'il te plaît. Voilà. Victorina tend le fruit. Il est lisse et un peu froid. Merci, marchande. Et moi, le sac ? Aniss tient le panier. Victorina pose l'orange dedans. La guêpe s'éloigne de l'écorce.</t>
+          <t>Victorina avance trop vite vers le papier. Tu mets l'enseigne, maintenant ! Les mots se bousculent dans sa bouche. Non. Aniss reste près du mur. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle pose le papier, un peu. Le papier est par terre, Victorina ? Papa reste à sa hauteur. Les caisses sont chaudes, sous tes mains. Tu veux la boutique ? Aniss ne dit rien. Il regarde le haut de la pile. Je regarde. D'accord. Merci, Victorina. Papa a entendu toute la phrase. Tu tiens le papier des deux mains ? Oui, maman. L'orange est penchée. Tu parles du store, si tu veux ? Le store claque un peu. On reste dans la cour, Victorina ? Oui. Aniss tend le bras, sans presser. Il pose le papier sur la caisse. L'orange dessinée regarde la cour. La boutique est ouverte ! Elle est en haut. Moi, le comptoir. Victorina s'assoit derrière la petite caisse. Elle aligne les trois oranges. Une orange, s'il te plaît. Voilà. Victorina tend le fruit. Il est lisse et un peu froid. Tu as les mains au frais ? Un peu, maman. La peau est lisse. Tu la mets dans le panier ? Celle du comptoir. Victorina pose une main sur l'orange. Le fruit colle un peu aux doigts.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss tend le bras. Il pose le papier sur la caisse. L'orange dessinée regarde la cour. La boutique est ouverte ! Bravo, Aniss. Tu as mis l'enseigne. Victorina s'assoit derrière la petite caisse. C'est le comptoir. Elle aligne les trois oranges. Une orange roule sous la pile. Elle est partie. Je ne la vois plus. Victorina se glisse près du bois. Elle est plus petite. Elle attrape l'orange. Te voilà. Chacun aide, à sa taille. Vous jouez ensemble. Maman prend une pièce imaginaire. Une orange, s'il te plaît. Voilà. Victorina tend le fruit. Il est lisse et un peu froid. Merci, marchande. Et moi, le sac ? Aniss tient le panier. Victorina pose l'orange dedans. La guêpe s'éloigne de l'écorce.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina avance trop vite vers le papier. Tu mets l'enseigne, maintenant ! Les mots se bousculent dans sa bouche. Non. Aniss reste près du mur. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle pose le papier, un peu. Le papier est par terre, Victorina ? Papa reste à sa hauteur. Les caisses sont chaudes, sous tes mains. &lt;emphasis level="moderate"&gt;Tu veux la boutique&lt;/emphasis&gt; ? Aniss ne dit rien. Il regarde le haut de la pile. Je regarde. D'accord. Merci, Victorina. Papa a entendu toute la phrase. Tu tiens le papier des deux mains ? Oui, maman. L'orange est penchée. Tu parles du store, si tu veux ? Le store claque un peu. On reste dans la cour, Victorina ? Oui. Aniss tend le bras, sans presser. Il pose le papier sur la caisse. L'orange dessinée regarde la cour. La boutique est ouverte ! Elle est en haut. Moi, le comptoir. Victorina s'assoit derrière la petite caisse. Elle aligne les trois oranges. Une orange, s'il te plaît. Voilà. Victorina tend le fruit. Il est lisse et un peu froid. Tu as les mains au frais ? Un peu, maman. La peau est lisse. Tu la mets dans le panier ? Celle du comptoir. Victorina pose une main sur l'orange. Le fruit colle un peu aux doigts.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Coralie a invité. Hippolyte a dit oui. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils jouent ensemble. [pause]</t>
+          <t>Victorina avance trop vite vers le papier. Tu mets l'enseigne, maintenant ! Les mots se bousculent dans sa bouche. Non. Aniss reste près du mur. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle pose le papier, un peu. Le papier est par terre, Victorina ? Papa reste à sa hauteur. Les caisses sont chaudes, sous tes mains. &lt;emphasis&gt;Tu veux la boutique&lt;/emphasis&gt; ? Aniss ne dit rien. Il regarde le haut de la pile. Je regarde. D'accord. Merci, Victorina. Papa a entendu toute la phrase. Tu tiens le papier des deux mains ? Oui, maman. L'orange est penchée. Tu parles du store, si tu veux ? Le store claque un peu. On reste dans la cour, Victorina ? Oui. Aniss tend le bras, sans presser. Il pose le papier sur la caisse. L'orange dessinée regarde la cour. La boutique est ouverte ! Elle est en haut. Moi, le comptoir. Victorina s'assoit derrière la petite caisse. Elle aligne les trois oranges. Une orange, s'il te plaît. Voilà. Victorina tend le fruit. Il est lisse et un peu froid. Tu as les mains au frais ? Un peu, maman. La peau est lisse. Tu la mets dans le panier ? Celle du comptoir. Victorina pose une main sur l'orange. Le fruit colle un peu aux doigts. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1640,7 +1657,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1648,10 +1665,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1674,30 +1691,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>Tu veux la boutique</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1706,10 +1723,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,39 +1739,61 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_invite_aniss_regarde; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss tend le bras.
+          <t>narrateur|Victorina avance trop vite vers le papier.
+enfant-f|Tu mets l'enseigne, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Non.
+narrateur|Aniss reste près du mur.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorina refuse de foncer.
+narrateur|Elle pose le papier, un peu.
+papa|Le papier est par terre, Victorina ?
+narrateur|Papa reste à sa hauteur.
+maman|Les caisses sont chaudes, sous tes mains.
+enfant-f|Tu veux la boutique ?
+narrateur|Aniss ne dit rien.
+narrateur|Il regarde le haut de la pile.
+copain|Je regarde.
+enfant-f|D'accord.
+papa|Merci, Victorina.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu tiens le papier des deux mains ?
+enfant-f|Oui, maman.
+enfant-f|L'orange est penchée.
+papa|Tu parles du store, si tu veux ?
+enfant-f|Le store claque un peu.
+maman|On reste dans la cour, Victorina ?
+enfant-f|Oui.
+narrateur|Aniss tend le bras, sans presser.
 narrateur|Il pose le papier sur la caisse.
 narrateur|L'orange dessinée regarde la cour.
 enfant-f|La boutique est ouverte !
-maman|Bravo, Aniss.
-maman|Tu as mis l'enseigne.
+copain|Elle est en haut.
+enfant-f|Moi, le comptoir.
 narrateur|Victorina s'assoit derrière la petite caisse.
-narrateur|C'est le comptoir.
 narrateur|Elle aligne les trois oranges.
-narrateur|Une orange roule sous la pile.
-enfant-f|Elle est partie.
-copain|Je ne la vois plus.
-narrateur|Victorina se glisse près du bois.
-narrateur|Elle est plus petite.
-narrateur|Elle attrape l'orange.
-enfant-f|Te voilà.
-maman|Chacun aide, à sa taille.
-maman|Vous jouez ensemble.
-narrateur|Maman prend une pièce imaginaire.
-maman|Une orange, s'il te plaît.
+papa|Une orange, s'il te plaît.
 enfant-f|Voilà.
 narrateur|Victorina tend le fruit.
 narrateur|Il est lisse et un peu froid.
-maman|Merci, marchande.
-copain|Et moi, le sac ?
-narrateur|Aniss tient le panier.
-narrateur|Victorina pose l'orange dedans.
-narrateur|La guêpe s'éloigne de l'écorce.</t>
+maman|Tu as les mains au frais ?
+enfant-f|Un peu, maman.
+enfant-f|La peau est lisse.
+papa|Tu la mets dans le panier ?
+enfant-f|Celle du comptoir.
+narrateur|Victorina pose une main sur l'orange.
+narrateur|Le fruit colle un peu aux doigts.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>orange</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On ferme la boutique ? Encore un client. Moi. Aniss achète la dernière orange. Il fait semblant de croquer. Elle est sucrée. C'est la plus belle. Vous avez des tailles différentes. Et vous avez joué ensemble. Victorina range le papier dans la caisse. Aniss empile le bois. Tu as fini de ranger le papier ? Oui, maman. L'ombre du figuier a bougé. La tache de figue est encore là.</t>
+          <t>Victorina pousse une orange trop vite. La dernière, maintenant ! L'orange roule sous la pile. Oh. Je ne la vois plus. Aniss se baisse, trop grand. Son épaule tape le bois. Oh. Papa n'a pas fini sa phrase. L'orange file, Victorina. Les deux voix se mélangent. Oh. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cour, un instant. Elle observe le bois, écoute le store. Sur la pierre, un éclat de figue luit. Il est là. Tu tiens la pile, si tu veux ? Oui. Aniss tient la grande caisse. Victorina se glisse près du bois. Elle attrape l'orange. Te voilà. Tu restes un peu ? Oui, papa. Le panier est près du mur. Et moi, le sac ? Aniss tient le panier. Victorina pose l'orange dedans. Elle est à nous. Elle est dans le panier. Je la tiens bien. On marche. Le panier penche, puis se cale. Je la tiens. On avance.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On ferme la boutique ? Encore un client. Moi. Aniss achète la dernière orange. Il fait semblant de croquer. Elle est sucrée. C'est la plus belle. Vous avez des tailles différentes. Et vous avez joué ensemble. Victorina range le papier dans la caisse. Aniss empile le bois. Tu as fini de ranger le papier ? Oui, maman. L'ombre du figuier a bougé. La tache de figue est encore là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina pousse une orange trop vite. La dernière, maintenant ! L'orange roule sous la pile. Oh. Je ne la vois plus. Aniss se baisse, trop grand. Son épaule tape le bois. Oh. Papa n'a pas fini sa phrase. L'orange file, Victorina. Les deux voix se mélangent. Oh. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cour, un instant. Elle observe le bois, écoute le store. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de figue&lt;/emphasis&gt; luit. Il est là. Tu tiens la pile, si tu veux ? Oui. Aniss tient la grande caisse. Victorina se glisse près du bois. Elle attrape l'orange. Te voilà. Tu restes un peu ? Oui, papa. Le panier est près du mur. Et moi, le sac ? Aniss tient le panier. Victorina pose l'orange dedans. Elle est à nous. Elle est dans le panier. Je la tiens bien. On marche. Le panier penche, puis se cale. Je la tiens. On avance.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman dit : on range. Coralie range un seau. Hippolyte range une pelle. [pause]</t>
+          <t>Victorina pousse une orange trop vite. La dernière, maintenant ! L'orange roule sous la pile. Oh. Je ne la vois plus. Aniss se baisse, trop grand. Son épaule tape le bois. Oh. Papa n'a pas fini sa phrase. L'orange file, Victorina. Les deux voix se mélangent. Oh. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cour, un instant. Elle observe le bois, écoute le store. Sur la pierre, un &lt;emphasis&gt;éclat de figue&lt;/emphasis&gt; luit. Il est là. Tu tiens la pile, si tu veux ? Oui. Aniss tient la grande caisse. Victorina se glisse près du bois. Elle attrape l'orange. Te voilà. Tu restes un peu ? Oui, papa. Le panier est près du mur. Et moi, le sac ? Aniss tient le panier. Victorina pose l'orange dedans. Elle est à nous. Elle est dans le panier. Je la tiens bien. On marche. Le panier penche, puis se cale. Je la tiens. On avance. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de figue</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1914,24 +1957,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sous_la_pile; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On ferme la boutique ?
-enfant-f|Encore un client.
-copain|Moi.
-narrateur|Aniss achète la dernière orange.
-narrateur|Il fait semblant de croquer.
-copain|Elle est sucrée.
-enfant-f|C'est la plus belle.
-maman|Vous avez des tailles différentes.
-maman|Et vous avez joué ensemble.
-narrateur|Victorina range le papier dans la caisse.
-narrateur|Aniss empile le bois.
-maman|Tu as fini de ranger le papier ?
-enfant-f|Oui, maman.
-narrateur|L'ombre du figuier a bougé.
-narrateur|La tache de figue est encore là.</t>
+          <t>narrateur|Victorina pousse une orange trop vite.
+enfant-f|La dernière, maintenant !
+narrateur|L'orange roule sous la pile.
+enfant-f|Oh.
+copain|Je ne la vois plus.
+narrateur|Aniss se baisse, trop grand.
+narrateur|Son épaule tape le bois.
+enfant-f|Oh.
+narrateur|Papa n'a pas fini sa phrase.
+papa|L'orange file, Victorina.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Victorina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute la cour, un instant.
+narrateur|Elle observe le bois, écoute le store.
+narrateur|Sur la pierre, un éclat de figue luit.
+enfant-f|Il est là.
+enfant-f|Tu tiens la pile, si tu veux ?
+copain|Oui.
+narrateur|Aniss tient la grande caisse.
+narrateur|Victorina se glisse près du bois.
+narrateur|Elle attrape l'orange.
+enfant-f|Te voilà.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Le panier est près du mur.
+copain|Et moi, le sac ?
+narrateur|Aniss tient le panier.
+narrateur|Victorina pose l'orange dedans.
+enfant-f|Elle est à nous.
+maman|Elle est dans le panier.
+enfant-f|Je la tiens bien.
+papa|On marche.
+narrateur|Le panier penche, puis se cale.
+enfant-f|Je la tiens.
+maman|On avance.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>bois</t>
         </is>
       </c>
     </row>
@@ -1958,17 +2032,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a ouvert la boutique. L'enseigne était en haut. Vous avez joué ensemble. La cour sent encore l'orange.</t>
+          <t>La figue brillait, papa. Tu le vois, comme dans la cour ? Oui, sur la pierre. Victorina pose le panier contre elle. On la garde au frais ? Oui, maman. Les oranges sentaient bon. Elle est contre toi. Une odeur d'orange monte du panier. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. On le voit, maman. Tu le vois sur la pierre ? Oui, l'éclat. Un éclat de figue reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a ouvert la boutique. L'enseigne était en haut. Vous avez joué ensemble. La cour sent encore l'orange.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La figue brillait, papa. Tu le vois, comme dans la cour ? Oui, sur la pierre. Victorina pose le panier contre elle. On la garde au frais ? Oui, maman. Les oranges sentaient bon. Elle est contre toi. Une odeur d'orange monte du panier. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. On le voit, maman. Tu le vois sur la pierre ? Oui, l'éclat. Un &lt;emphasis level="moderate"&gt;éclat de figue&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La figue brillait, papa. Tu le vois, comme dans la cour ? Oui, sur la pierre. Victorina pose le panier contre elle. On la garde au frais ? Oui, maman. Les oranges sentaient bon. Elle est contre toi. Une odeur d'orange monte du panier. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. On le voit, maman. Tu le vois sur la pierre ? Oui, l'éclat. Un &lt;emphasis&gt;éclat de figue&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2015,7 +2089,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2023,10 +2097,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2035,12 +2109,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2049,17 +2123,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de figue</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2068,11 +2146,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2081,27 +2159,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|On a ouvert la boutique.
-copain|L'enseigne était en haut.
-maman|Vous avez joué ensemble.
-narrateur|La cour sent encore l'orange.</t>
+          <t>enfant-f|La figue brillait, papa.
+papa|Tu le vois, comme dans la cour ?
+enfant-f|Oui, sur la pierre.
+narrateur|Victorina pose le panier contre elle.
+maman|On la garde au frais ?
+enfant-f|Oui, maman.
+enfant-f|Les oranges sentaient bon.
+maman|Elle est contre toi.
+narrateur|Une odeur d'orange monte du panier.
+narrateur|Victorina respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Victorina se réchauffent.
+enfant-f|On le voit, maman.
+maman|Tu le vois sur la pierre ?
+enfant-f|Oui, l'éclat.
+narrateur|Un éclat de figue reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>figue</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2307,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>